<commit_message>
Add R1 stage 4: PLZ store selection and path without store
OpenGeoDB PLZ reference table, code-side PLZ check, stores sorted by
distance and never selected automatically, list with change/add store.
Triggered by the stage-4 request (OpenGeoDB, 50 km, 5 stores confirmed).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EimuL5ZzreqsH6e3579jk7
</commit_message>
<xml_diff>
--- a/app/data/baumarkt-buddy-data.xlsx
+++ b/app/data/baumarkt-buddy-data.xlsx
@@ -6202,10 +6202,10 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>52.517</v>
+        <v>52.5167</v>
       </c>
       <c r="F2" t="n">
-        <v>13.3889</v>
+        <v>13.4</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -6235,10 +6235,10 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>48.1374</v>
+        <v>48.15</v>
       </c>
       <c r="F3" t="n">
-        <v>11.5755</v>
+        <v>11.5833</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -6268,10 +6268,10 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>53.5503</v>
+        <v>53.5489</v>
       </c>
       <c r="F4" t="n">
-        <v>10.0006</v>
+        <v>10.00574</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>

</xml_diff>